<commit_message>
Clarify Stage 4 agent-level framing
</commit_message>
<xml_diff>
--- a/analysis(S4)/tables/level2_agent_network_analysis.xlsx
+++ b/analysis(S4)/tables/level2_agent_network_analysis.xlsx
@@ -131,13 +131,13 @@
     <t>level2_core_no_article_count</t>
   </si>
   <si>
-    <t>level2_mechanism_centrality</t>
-  </si>
-  <si>
-    <t>level2_mechanism_repeat_exposure</t>
-  </si>
-  <si>
-    <t>level2_mechanism_network_composition</t>
+    <t>level2_descriptor_centrality</t>
+  </si>
+  <si>
+    <t>level2_descriptor_repeat_exposure</t>
+  </si>
+  <si>
+    <t>level2_descriptor_network_composition</t>
   </si>
   <si>
     <t>ols</t>
@@ -260,7 +260,7 @@
     <t>status</t>
   </si>
   <si>
-    <t>level2_mechanism_predictors</t>
+    <t>level2_descriptor_variables</t>
   </si>
   <si>
     <t>log_article_count_per_agent, agent_deg_centrality_mean, avg_out_degree_centrality_mean, repeat_exposure_1st_nodes_pct, repeat_exposure_2nd_nodes_pct, gender_assortativity_mean</t>

</xml_diff>